<commit_message>
Update filters and companies: add Cupertino, SDE role, company list
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Preferred_Companies.xlsx
+++ b/data/Preferred_Companies.xlsx
@@ -1,21 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nived\Projects\JobScraper\JobScraper\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD295922-A216-4F59-A3F4-D8D5BB3D6870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="22932" yWindow="972" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Companies" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Companies" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -37,18 +28,6 @@
     <t>https://stripe.com/jobs</t>
   </si>
   <si>
-    <t>OpenAI</t>
-  </si>
-  <si>
-    <t>https://openai.com/careers/</t>
-  </si>
-  <si>
-    <t>Anthropic</t>
-  </si>
-  <si>
-    <t>https://www.anthropic.com/careers</t>
-  </si>
-  <si>
     <t>Palantir</t>
   </si>
   <si>
@@ -64,115 +43,127 @@
     <t>Fireworks AI</t>
   </si>
   <si>
+    <t>https://fireworks.ai/careers</t>
+  </si>
+  <si>
     <t>Everpure Inc.</t>
   </si>
   <si>
+    <t>https://www.everpuredata.com/company/careers/opportunities.html#engineering&amp;united-states&amp;</t>
+  </si>
+  <si>
     <t>Databricks</t>
   </si>
   <si>
+    <t>https://www.databricks.com/company/careers/open-positions</t>
+  </si>
+  <si>
     <t>Uber</t>
   </si>
   <si>
+    <t>https://jobs.uber.com/en/jobs/?team=Engineer</t>
+  </si>
+  <si>
     <t>Giga</t>
   </si>
   <si>
+    <t>https://jobs.ashbyhq.com/gigaml</t>
+  </si>
+  <si>
     <t>Ramp</t>
   </si>
   <si>
+    <t>https://jobs.ashbyhq.com/ramp</t>
+  </si>
+  <si>
     <t>Gemini</t>
   </si>
   <si>
+    <t>https://www.gemini.com/careers#open-roles</t>
+  </si>
+  <si>
     <t>Sentry</t>
   </si>
   <si>
+    <t>https://jobs.ashbyhq.com/sentry?original_referrer=https%3A%2F%2Fsentry.io%2Fcareers%2F</t>
+  </si>
+  <si>
     <t>Datadog</t>
   </si>
   <si>
+    <t>https://careers.datadoghq.com/all-jobs/</t>
+  </si>
+  <si>
     <t>Snowflake</t>
   </si>
   <si>
+    <t>https://careers.snowflake.com/us/en/c/engineering-jobs</t>
+  </si>
+  <si>
     <t>MongoDB</t>
   </si>
   <si>
+    <t>https://www.mongodb.com/company/careers/teams/engineering</t>
+  </si>
+  <si>
     <t>EliseAI</t>
   </si>
   <si>
+    <t>https://jobs.ashbyhq.com/eliseai</t>
+  </si>
+  <si>
     <t>Notion</t>
   </si>
   <si>
+    <t>https://www.notion.com/careers</t>
+  </si>
+  <si>
+    <t>Rippling</t>
+  </si>
+  <si>
+    <t>https://www.rippling.com/careers/open-roles?department=Engineering&amp;location=San%20Francisco%2C%20CA</t>
+  </si>
+  <si>
     <t>Figma</t>
   </si>
   <si>
+    <t>https://www.figma.com/careers/</t>
+  </si>
+  <si>
     <t>Adobe</t>
   </si>
   <si>
+    <t>https://research.adobe.com/careers/, https://careers.adobe.com/us/en/c/engineering-and-product-jobs</t>
+  </si>
+  <si>
     <t>CrewAI</t>
   </si>
   <si>
     <t>https://apply.workable.com/crewai/?lng=en</t>
   </si>
   <si>
-    <t>https://research.adobe.com/careers/, https://careers.adobe.com/us/en/c/engineering-and-product-jobs</t>
-  </si>
-  <si>
-    <t>https://www.figma.com/careers/</t>
-  </si>
-  <si>
-    <t>https://www.notion.com/careers</t>
-  </si>
-  <si>
-    <t>https://jobs.ashbyhq.com/eliseai</t>
-  </si>
-  <si>
-    <t>https://www.mongodb.com/company/careers/teams/engineering</t>
-  </si>
-  <si>
-    <t>https://careers.snowflake.com/us/en/c/engineering-jobs</t>
-  </si>
-  <si>
-    <t>https://careers.datadoghq.com/all-jobs/</t>
-  </si>
-  <si>
-    <t>https://jobs.ashbyhq.com/sentry?original_referrer=https%3A%2F%2Fsentry.io%2Fcareers%2F</t>
-  </si>
-  <si>
-    <t>https://www.gemini.com/careers#open-roles</t>
-  </si>
-  <si>
-    <t>https://jobs.ashbyhq.com/ramp</t>
-  </si>
-  <si>
-    <t>https://jobs.ashbyhq.com/gigaml</t>
-  </si>
-  <si>
-    <t>https://jobs.uber.com/en/jobs/?team=Engineer</t>
-  </si>
-  <si>
-    <t>https://fireworks.ai/careers</t>
-  </si>
-  <si>
-    <t>https://www.databricks.com/company/careers/open-positions</t>
-  </si>
-  <si>
-    <t>https://www.everpuredata.com/company/careers/opportunities.html#engineering&amp;united-states&amp;</t>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>https://jobs.apple.com/en-us/search?search=software+engineer&amp;sort=newest&amp;location=cupertino-CUP+sunnyvale-SVL&amp;page=16&amp;key=software&amp;team=machine-learning-infrastructure-MLAI-MLI+deep-learning-and-reinforcement-learning-MLAI-DLRL+natural-language-processing-and-speech-technologies-MLAI-NLP+computer-vision-MLAI-CV+applied-research-MLAI-AR+apps-and-frameworks-SFTWR-AF+cloud-and-infrastructure-SFTWR-CLD+core-operating-systems-SFTWR-COS+devops-and-site-reliability-SFTWR-DSR+engineering-project-management-SFTWR-EPM+information-systems-and-technology-SFTWR-ISTECH+machine-learning-and-ai-SFTWR-MCHLN+security-and-privacy-SFTWR-SEC+software-quality-automation-and-tools-SFTWR-SQAT+wireless-software-SFTWR-WSFT+information-systems-and-technology-CORSV-IT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -186,7 +177,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF4472C4"/>
-        <bgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -212,7 +202,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -299,6 +289,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -333,6 +324,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -367,20 +359,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -502,19 +490,59 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="41" customWidth="1"/>
-    <col min="3" max="3" width="53" customWidth="1"/>
+    <col min="3" max="3" width="42.142857142857146" customWidth="1"/>
+    <col min="4" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -528,7 +556,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -536,7 +564,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -544,7 +572,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -552,7 +580,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -560,7 +588,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -568,89 +596,89 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
         <v>34</v>
@@ -658,45 +686,46 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B22" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>